<commit_message>
Fix non-deterministic expiry tie-break in Rust engine; correct 24-month results
The Rust engine built its per-day expiry list from a HashSet without
sorting, so when two expiries were equally far from the target DTE it
picked one at random per process. On 2025-09-24 (20 Oct vs 28 Oct 2025)
identical reruns gave 12 trades or 11. Expiries are now sorted, matching
the Python engine. Verified: 8/8 fresh runs on the 24-month data agree
with Python (11 trades, Rs 4,91,765); both 10-month windows also match.

Corrected headline: 11 trades, 54.5% win rate, -1.65% return, Sharpe -0.13,
max drawdown -3.17%, profit factor 0.74 (was 12 / 58.3% / -1.29%).
Regenerated results workbook, charts, and report PDF. README and
README_RUST now state that Rust is not faster here (0.8 s Python vs 3.7 s
Rust end to end, dominated by list conversion) instead of implying it is.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results_24m.xlsx
+++ b/results_24m.xlsx
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>-1.29</v>
+        <v>-1.65</v>
       </c>
     </row>
     <row r="4">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>58.33</v>
+        <v>54.55</v>
       </c>
     </row>
     <row r="5">
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>-3.16</v>
+        <v>-3.17</v>
       </c>
     </row>
     <row r="6">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>-0.09</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="7">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>0.8</v>
+        <v>0.74</v>
       </c>
     </row>
     <row r="8">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>493535</v>
+        <v>491765</v>
       </c>
     </row>
   </sheetData>
@@ -541,7 +541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -854,40 +854,40 @@
     </row>
     <row r="6">
       <c r="A6" s="6" t="n">
-        <v>45924</v>
+        <v>45985</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>45936</v>
+        <v>45993</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>45958</v>
+        <v>46014</v>
       </c>
       <c r="D6" t="n">
-        <v>25800</v>
+        <v>26750</v>
       </c>
       <c r="E6" t="n">
-        <v>24300</v>
+        <v>25200</v>
       </c>
       <c r="F6" t="n">
-        <v>26000</v>
+        <v>26900</v>
       </c>
       <c r="G6" t="n">
-        <v>24100</v>
+        <v>25000</v>
       </c>
       <c r="H6" t="n">
-        <v>45.69999999999999</v>
+        <v>63.49999999999999</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>3427.499999999999</v>
+        <v>4762.499999999999</v>
       </c>
       <c r="J6" t="n">
-        <v>22.09999999999999</v>
+        <v>30.65000000000001</v>
       </c>
       <c r="K6" t="n">
-        <v>23.59999999999999</v>
+        <v>32.84999999999998</v>
       </c>
       <c r="L6" s="5" t="n">
-        <v>1770</v>
+        <v>2463.749999999999</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -895,377 +895,325 @@
         </is>
       </c>
       <c r="N6" s="5" t="n">
-        <v>504173.75</v>
+        <v>504867.5</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0.35</v>
+        <v>0.49</v>
       </c>
       <c r="P6" s="3" t="n">
-        <v>0.83</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
-        <v>45985</v>
+        <v>46034</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>45993</v>
+        <v>46036</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>46014</v>
+        <v>46063</v>
       </c>
       <c r="D7" t="n">
+        <v>26550</v>
+      </c>
+      <c r="E7" t="n">
+        <v>25000</v>
+      </c>
+      <c r="F7" t="n">
         <v>26750</v>
       </c>
-      <c r="E7" t="n">
-        <v>25200</v>
-      </c>
-      <c r="F7" t="n">
-        <v>26900</v>
-      </c>
       <c r="G7" t="n">
-        <v>25000</v>
+        <v>24800</v>
       </c>
       <c r="H7" t="n">
-        <v>63.49999999999999</v>
+        <v>17.59999999999999</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>4762.499999999999</v>
+        <v>1320</v>
       </c>
       <c r="J7" t="n">
-        <v>30.65000000000001</v>
+        <v>55</v>
       </c>
       <c r="K7" t="n">
-        <v>32.84999999999998</v>
+        <v>-37.40000000000001</v>
       </c>
       <c r="L7" s="5" t="n">
-        <v>2463.749999999999</v>
+        <v>-2805</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>profit_target</t>
+          <t>stop_loss</t>
         </is>
       </c>
       <c r="N7" s="5" t="n">
-        <v>506637.5</v>
+        <v>502062.5</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>0.49</v>
+        <v>-0.5600000000000001</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>1.33</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
-        <v>46034</v>
+        <v>46041</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>46036</v>
+        <v>46056</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>46063</v>
+        <v>46070</v>
       </c>
       <c r="D8" t="n">
+        <v>26350</v>
+      </c>
+      <c r="E8" t="n">
+        <v>24900</v>
+      </c>
+      <c r="F8" t="n">
         <v>26550</v>
       </c>
-      <c r="E8" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F8" t="n">
-        <v>26750</v>
-      </c>
       <c r="G8" t="n">
-        <v>24800</v>
+        <v>24600</v>
       </c>
       <c r="H8" t="n">
-        <v>17.59999999999999</v>
+        <v>116.9</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>1320</v>
+        <v>8767.499999999998</v>
       </c>
       <c r="J8" t="n">
-        <v>55</v>
+        <v>39.65</v>
       </c>
       <c r="K8" t="n">
-        <v>-37.40000000000001</v>
+        <v>77.24999999999997</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>-2805</v>
+        <v>5793.749999999998</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>stop_loss</t>
+          <t>profit_target</t>
         </is>
       </c>
       <c r="N8" s="5" t="n">
-        <v>503832.5</v>
+        <v>507856.25</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>-0.5600000000000001</v>
+        <v>1.16</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>0.77</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
-        <v>46041</v>
+        <v>46066</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>46056</v>
+        <v>46092</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>46070</v>
+        <v>46098</v>
       </c>
       <c r="D9" t="n">
-        <v>26350</v>
+        <v>26300</v>
       </c>
       <c r="E9" t="n">
-        <v>24900</v>
+        <v>24700</v>
       </c>
       <c r="F9" t="n">
-        <v>26550</v>
+        <v>26500</v>
       </c>
       <c r="G9" t="n">
-        <v>24600</v>
+        <v>24500</v>
       </c>
       <c r="H9" t="n">
-        <v>116.9</v>
+        <v>49.75</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>8767.499999999998</v>
+        <v>3731.25</v>
       </c>
       <c r="J9" t="n">
-        <v>39.65</v>
+        <v>164.9</v>
       </c>
       <c r="K9" t="n">
-        <v>77.24999999999997</v>
+        <v>-115.15</v>
       </c>
       <c r="L9" s="5" t="n">
-        <v>5793.749999999998</v>
+        <v>-8636.249999999998</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>profit_target</t>
+          <t>stop_loss</t>
         </is>
       </c>
       <c r="N9" s="5" t="n">
-        <v>509626.25</v>
+        <v>499220</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>1.16</v>
+        <v>-1.73</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>1.93</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
-        <v>46066</v>
+        <v>46125</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>46092</v>
+        <v>46147</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>46098</v>
+        <v>46154</v>
       </c>
       <c r="D10" t="n">
-        <v>26300</v>
+        <v>24600</v>
       </c>
       <c r="E10" t="n">
-        <v>24700</v>
+        <v>23000</v>
       </c>
       <c r="F10" t="n">
-        <v>26500</v>
+        <v>24800</v>
       </c>
       <c r="G10" t="n">
-        <v>24500</v>
+        <v>22950</v>
       </c>
       <c r="H10" t="n">
-        <v>49.75</v>
+        <v>80.45000000000005</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>3731.25</v>
+        <v>6033.750000000004</v>
       </c>
       <c r="J10" t="n">
-        <v>164.9</v>
+        <v>23</v>
       </c>
       <c r="K10" t="n">
-        <v>-115.15</v>
+        <v>57.45000000000005</v>
       </c>
       <c r="L10" s="5" t="n">
-        <v>-8636.249999999998</v>
+        <v>4308.750000000004</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>stop_loss</t>
+          <t>profit_target</t>
         </is>
       </c>
       <c r="N10" s="5" t="n">
-        <v>500990</v>
+        <v>503528.75</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>-1.73</v>
+        <v>0.86</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>0.2</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
-        <v>46125</v>
+        <v>46178</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>46147</v>
+        <v>46210</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>46154</v>
+        <v>46210</v>
       </c>
       <c r="D11" t="n">
-        <v>24600</v>
+        <v>24050</v>
       </c>
       <c r="E11" t="n">
-        <v>23000</v>
+        <v>22650</v>
       </c>
       <c r="F11" t="n">
-        <v>24800</v>
+        <v>24250</v>
       </c>
       <c r="G11" t="n">
-        <v>22950</v>
+        <v>22400</v>
       </c>
       <c r="H11" t="n">
-        <v>80.45000000000005</v>
+        <v>81.40000000000003</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>6033.750000000004</v>
+        <v>6105.000000000003</v>
       </c>
       <c r="J11" t="n">
-        <v>23</v>
+        <v>200</v>
       </c>
       <c r="K11" t="n">
-        <v>57.45000000000005</v>
+        <v>-118.6</v>
       </c>
       <c r="L11" s="5" t="n">
-        <v>4308.750000000004</v>
+        <v>-8894.999999999998</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>profit_target</t>
+          <t>expiry</t>
         </is>
       </c>
       <c r="N11" s="5" t="n">
-        <v>505298.75</v>
+        <v>494633.75</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>0.86</v>
+        <v>-1.78</v>
       </c>
       <c r="P11" s="3" t="n">
-        <v>1.06</v>
+        <v>-1.07</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
-        <v>46178</v>
+        <v>46237</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>46210</v>
+        <v>46238</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>46210</v>
+        <v>46266</v>
       </c>
       <c r="D12" t="n">
-        <v>24050</v>
+        <v>25550</v>
       </c>
       <c r="E12" t="n">
-        <v>22650</v>
+        <v>24000</v>
       </c>
       <c r="F12" t="n">
-        <v>24250</v>
+        <v>25700</v>
       </c>
       <c r="G12" t="n">
-        <v>22400</v>
+        <v>23800</v>
       </c>
       <c r="H12" t="n">
-        <v>81.40000000000003</v>
+        <v>6.299999999999997</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>6105.000000000003</v>
+        <v>472.4999999999998</v>
       </c>
       <c r="J12" t="n">
-        <v>200</v>
+        <v>44.55000000000001</v>
       </c>
       <c r="K12" t="n">
-        <v>-118.6</v>
+        <v>-38.25000000000001</v>
       </c>
       <c r="L12" s="5" t="n">
-        <v>-8894.999999999998</v>
+        <v>-2868.750000000001</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>expiry</t>
+          <t>stop_loss</t>
         </is>
       </c>
       <c r="N12" s="5" t="n">
-        <v>496403.75</v>
+        <v>491765</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>-1.78</v>
+        <v>-0.57</v>
       </c>
       <c r="P12" s="3" t="n">
-        <v>-0.72</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="n">
-        <v>46237</v>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>46238</v>
-      </c>
-      <c r="C13" s="6" t="n">
-        <v>46266</v>
-      </c>
-      <c r="D13" t="n">
-        <v>25550</v>
-      </c>
-      <c r="E13" t="n">
-        <v>24000</v>
-      </c>
-      <c r="F13" t="n">
-        <v>25700</v>
-      </c>
-      <c r="G13" t="n">
-        <v>23800</v>
-      </c>
-      <c r="H13" t="n">
-        <v>6.299999999999997</v>
-      </c>
-      <c r="I13" s="5" t="n">
-        <v>472.4999999999998</v>
-      </c>
-      <c r="J13" t="n">
-        <v>44.55000000000001</v>
-      </c>
-      <c r="K13" t="n">
-        <v>-38.25000000000001</v>
-      </c>
-      <c r="L13" s="5" t="n">
-        <v>-2868.750000000001</v>
-      </c>
-      <c r="M13" t="inlineStr">
-        <is>
-          <t>stop_loss</t>
-        </is>
-      </c>
-      <c r="N13" s="5" t="n">
-        <v>493535</v>
-      </c>
-      <c r="O13" s="3" t="n">
-        <v>-0.57</v>
-      </c>
-      <c r="P13" s="3" t="n">
-        <v>-1.29</v>
+        <v>-1.65</v>
       </c>
     </row>
   </sheetData>
@@ -1279,7 +1227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1350,90 +1298,79 @@
     </row>
     <row r="6">
       <c r="A6" s="7" t="n">
-        <v>45936</v>
+        <v>45993</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>504173.75</v>
+        <v>504867.5</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.83</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="n">
-        <v>45993</v>
+        <v>46036</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>506637.5</v>
+        <v>502062.5</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>1.33</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="n">
-        <v>46036</v>
+        <v>46056</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>503832.5</v>
+        <v>507856.25</v>
       </c>
       <c r="C8" s="3" t="n">
-        <v>0.77</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="n">
-        <v>46056</v>
+        <v>46092</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>509626.25</v>
+        <v>499220</v>
       </c>
       <c r="C9" s="3" t="n">
-        <v>1.93</v>
+        <v>-0.16</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="n">
-        <v>46092</v>
+        <v>46147</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>500990</v>
+        <v>503528.75</v>
       </c>
       <c r="C10" s="3" t="n">
-        <v>0.2</v>
+        <v>0.71</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="n">
-        <v>46147</v>
+        <v>46210</v>
       </c>
       <c r="B11" s="5" t="n">
-        <v>505298.75</v>
+        <v>494633.75</v>
       </c>
       <c r="C11" s="3" t="n">
-        <v>1.06</v>
+        <v>-1.07</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="n">
-        <v>46210</v>
+        <v>46238</v>
       </c>
       <c r="B12" s="5" t="n">
-        <v>496403.75</v>
+        <v>491765</v>
       </c>
       <c r="C12" s="3" t="n">
-        <v>-0.72</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="7" t="n">
-        <v>46238</v>
-      </c>
-      <c r="B13" s="5" t="n">
-        <v>493535</v>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>-1.29</v>
+        <v>-1.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>